<commit_message>
Replace Nelson (2005) citations with GSWA Geochronology Database
The six Leeuwin Inlier hornblende Ar–Ar entries cited Nelson (2005),
which does not contain those analyses. Source updated to GSWA
Geochronology Database, matching the manuscript citation.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/03_Data_Set_S1_Case_Study.xlsx
+++ b/03_Data_Set_S1_Case_Study.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lucymathieson/Desktop/leadloss-benchmark-manuscript-repro/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8C0777D-04FB-2E41-87B0-A866280A2CCE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D481EE7B-5303-E243-B1E1-3495389A2C09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5400" yWindow="660" windowWidth="29160" windowHeight="21680" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="528" uniqueCount="153">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="526" uniqueCount="150">
   <si>
     <t>Data Set S1</t>
   </si>
@@ -467,22 +467,13 @@
     <t>Wingate, M.T.D., Kirkland, C.L. &amp; Hall, C.E. (2011). 193435: biotite monzogranite, Police Road; Geochronology Record 960. Geological Survey of Western Australia.</t>
   </si>
   <si>
-    <t>Lu, S., Phillips, D., Kohn, B.P., Gleadow, A.J.W. &amp; Matchan, E.L. (2015). Thermotectonic evolution of the western margin of the Yilgarn craton, Western Australia: new insights from 40Ar/39Ar analysis of muscovite and biotite. Precambrian Research 270: 139-154. doi:10.1016/j.precamres.2015.09.005</t>
-  </si>
-  <si>
     <t>GSWA Geochronology database</t>
   </si>
   <si>
     <t>Geological Survey of Western Australia Geochronology database. Public geochronology and isotope data accessed via GeoVIEW.WA / GSWA Data and Software Centre.</t>
   </si>
   <si>
-    <t>Nelson (2005)</t>
-  </si>
-  <si>
-    <t>Nelson, D.R. (2005). 40Ar/39Ar hornblende cooling ages from the northern Leeuwin Complex (samples 112131, 112132, 112134, 112140, 112143, 112144A). Geochronology Records 599–604. Geological Survey of Western Australia, Perth. Accessed via GSWA Geochronology database, https://geoview.dmp.wa.gov.au/geoview/</t>
-  </si>
-  <si>
-    <t>Nelson (2005); GSWA Geochronology database</t>
+    <t>Lu, S., Phillips, D., Kohn, B.P., Gleadow, A.J.W. &amp; Matchan, E.L. (2015). Thermotectonic evolution of the western margin of the Yilgarn craton, Western Australia: new insights from 40Ar/39Ar analysis of muscovite and biotite. Precambrian Research 270: 139-154. 10.1016/j.precamres.2015.09.014</t>
   </si>
 </sst>
 </file>
@@ -1369,7 +1360,7 @@
         <v>114.98028100000001</v>
       </c>
       <c r="L9" t="s">
-        <v>152</v>
+        <v>147</v>
       </c>
     </row>
     <row r="10" spans="1:12" ht="16" customHeight="1" x14ac:dyDescent="0.2">
@@ -1407,7 +1398,7 @@
         <v>115.010161</v>
       </c>
       <c r="L10" t="s">
-        <v>152</v>
+        <v>147</v>
       </c>
     </row>
     <row r="11" spans="1:12" ht="16" customHeight="1" x14ac:dyDescent="0.2">
@@ -1445,7 +1436,7 @@
         <v>115.135811</v>
       </c>
       <c r="L11" t="s">
-        <v>152</v>
+        <v>147</v>
       </c>
     </row>
     <row r="12" spans="1:12" ht="16" customHeight="1" x14ac:dyDescent="0.2">
@@ -1483,7 +1474,7 @@
         <v>114.98731100000001</v>
       </c>
       <c r="L12" t="s">
-        <v>152</v>
+        <v>147</v>
       </c>
     </row>
     <row r="13" spans="1:12" ht="16" customHeight="1" x14ac:dyDescent="0.2">
@@ -1521,7 +1512,7 @@
         <v>115.02559100000001</v>
       </c>
       <c r="L13" t="s">
-        <v>152</v>
+        <v>147</v>
       </c>
     </row>
     <row r="14" spans="1:12" ht="16" customHeight="1" x14ac:dyDescent="0.2">
@@ -1559,7 +1550,7 @@
         <v>115.13600099999999</v>
       </c>
       <c r="L14" t="s">
-        <v>152</v>
+        <v>147</v>
       </c>
     </row>
     <row r="15" spans="1:12" ht="16" customHeight="1" x14ac:dyDescent="0.2">
@@ -3373,7 +3364,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="36" customWidth="1"/>
@@ -3390,10 +3381,10 @@
     </row>
     <row r="2" spans="1:2" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="B2" s="3" t="s">
         <v>148</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>149</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="32" customHeight="1" x14ac:dyDescent="0.2">
@@ -3409,36 +3400,28 @@
         <v>143</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="3" t="s">
-        <v>150</v>
+        <v>145</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" ht="32" customHeight="1" x14ac:dyDescent="0.2">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" ht="32" x14ac:dyDescent="0.2">
       <c r="A6" s="3" t="s">
-        <v>145</v>
+        <v>137</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" ht="32" x14ac:dyDescent="0.2">
-      <c r="A7" s="3" t="s">
-        <v>137</v>
-      </c>
-      <c r="B7" s="3" t="s">
         <v>144</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:B7">
-    <sortCondition ref="A1:A7"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:B6">
+    <sortCondition ref="A1:A6"/>
   </sortState>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>